<commit_message>
maybe fixed auto authentication. attempt at imlementing mock streamer
</commit_message>
<xml_diff>
--- a/screener/daily_screener_signals/2024-11-08.xlsx
+++ b/screener/daily_screener_signals/2024-11-08.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U39"/>
+  <dimension ref="A1:V36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -495,40 +495,45 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Yesterday High</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
           <t>Time Threshold</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Buy Time Threshold</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Sell_Time</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Market Cap</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Float</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Market Capitalization</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>Shares Float</t>
         </is>
@@ -576,38 +581,41 @@
         <v>0.3958346854202043</v>
       </c>
       <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr">
+      <c r="N2" t="n">
+        <v>0.4449</v>
+      </c>
+      <c r="O2" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P2" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q2" t="n">
+      <c r="R2" t="n">
         <v>10320000</v>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="S2" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="S2" t="n">
+      <c r="T2" t="n">
         <v>59080000</v>
       </c>
-      <c r="T2" t="inlineStr">
+      <c r="U2" t="inlineStr">
         <is>
           <t>10.32M</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
         <is>
           <t>59.08M</t>
         </is>
@@ -615,7 +623,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B3" t="n">
         <v>0</v>
@@ -629,16 +637,16 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>8.310596540956253</v>
+        <v>8.310164815699316</v>
       </c>
       <c r="F3" t="n">
-        <v>5.949668854826122</v>
+        <v>5.965978885287859</v>
       </c>
       <c r="G3" t="n">
         <v>0.09774436090225555</v>
       </c>
       <c r="H3" t="n">
-        <v>8.17</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -646,47 +654,50 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>127.5952929220153</v>
+        <v>127.6019216847224</v>
       </c>
       <c r="K3" t="n">
-        <v>9.141656195051878</v>
+        <v>9.141181297269249</v>
       </c>
       <c r="L3" t="n">
-        <v>7.89506671390844</v>
+        <v>7.89465657491435</v>
       </c>
       <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr">
+      <c r="N3" t="n">
+        <v>8.76</v>
+      </c>
+      <c r="O3" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P3" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>1025640000</v>
       </c>
-      <c r="R3" t="inlineStr">
+      <c r="S3" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="S3" t="n">
+      <c r="T3" t="n">
         <v>126170000</v>
       </c>
-      <c r="T3" t="inlineStr">
+      <c r="U3" t="inlineStr">
         <is>
           <t>1025.64M</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="V3" t="inlineStr">
         <is>
           <t>126.17M</t>
         </is>
@@ -694,7 +705,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B4" t="n">
         <v>0</v>
@@ -708,10 +719,10 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>1.039919225447168</v>
+        <v>1.039927867713707</v>
       </c>
       <c r="F4" t="n">
-        <v>5.109484191863794</v>
+        <v>5.513569988655076</v>
       </c>
       <c r="G4" t="n">
         <v>0.07000000000000006</v>
@@ -725,47 +736,50 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>1019.687850798247</v>
+        <v>1019.679376735317</v>
       </c>
       <c r="K4" t="n">
-        <v>1.143911147991884</v>
+        <v>1.143920654485078</v>
       </c>
       <c r="L4" t="n">
-        <v>0.9879232641748092</v>
+        <v>0.987931474328022</v>
       </c>
       <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr">
+      <c r="N4" t="n">
+        <v>1.07</v>
+      </c>
+      <c r="O4" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P4" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>121830000</v>
       </c>
-      <c r="R4" t="inlineStr">
+      <c r="S4" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="S4" t="n">
+      <c r="T4" t="n">
         <v>72650000</v>
       </c>
-      <c r="T4" t="inlineStr">
+      <c r="U4" t="inlineStr">
         <is>
           <t>121.83M</t>
         </is>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="V4" t="inlineStr">
         <is>
           <t>72.65M</t>
         </is>
@@ -773,7 +787,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B5" t="n">
         <v>0</v>
@@ -787,10 +801,10 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>129.9043110723513</v>
+        <v>129.9070661706564</v>
       </c>
       <c r="F5" t="n">
-        <v>7.048854829747564</v>
+        <v>7.070384739830859</v>
       </c>
       <c r="G5" t="n">
         <v>0.07840671369496471</v>
@@ -804,47 +818,50 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>8.162877669313106</v>
+        <v>8.162704549165801</v>
       </c>
       <c r="K5" t="n">
-        <v>142.8947421795865</v>
+        <v>142.8977727877221</v>
       </c>
       <c r="L5" t="n">
-        <v>123.4090955187338</v>
+        <v>123.4117128621236</v>
       </c>
       <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr">
+      <c r="N5" t="n">
+        <v>133.3</v>
+      </c>
+      <c r="O5" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P5" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>12141550000</v>
       </c>
-      <c r="R5" t="inlineStr">
+      <c r="S5" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="S5" t="n">
+      <c r="T5" t="n">
         <v>89520000</v>
       </c>
-      <c r="T5" t="inlineStr">
+      <c r="U5" t="inlineStr">
         <is>
           <t>12141.55M</t>
         </is>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="V5" t="inlineStr">
         <is>
           <t>89.52M</t>
         </is>
@@ -852,7 +869,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B6" t="n">
         <v>0</v>
@@ -866,10 +883,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2.528644405669419</v>
+        <v>2.531760980183811</v>
       </c>
       <c r="F6" t="n">
-        <v>7.882944618333907</v>
+        <v>7.800560494495192</v>
       </c>
       <c r="G6" t="n">
         <v>0.05645161290322586</v>
@@ -883,47 +900,50 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>419.3523603486974</v>
+        <v>418.8361414445267</v>
       </c>
       <c r="K6" t="n">
-        <v>2.781508846236361</v>
+        <v>2.784937078202192</v>
       </c>
       <c r="L6" t="n">
-        <v>2.402212185385948</v>
+        <v>2.40517293117462</v>
       </c>
       <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr">
+      <c r="N6" t="n">
+        <v>2.63</v>
+      </c>
+      <c r="O6" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P6" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q6" t="n">
+      <c r="R6" t="n">
         <v>1265780000</v>
       </c>
-      <c r="R6" t="inlineStr">
+      <c r="S6" t="inlineStr">
         <is>
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="S6" t="n">
+      <c r="T6" t="n">
         <v>524900000</v>
       </c>
-      <c r="T6" t="inlineStr">
+      <c r="U6" t="inlineStr">
         <is>
           <t>1265.78M</t>
         </is>
       </c>
-      <c r="U6" t="inlineStr">
+      <c r="V6" t="inlineStr">
         <is>
           <t>524.9M</t>
         </is>
@@ -931,7 +951,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B7" t="n">
         <v>0</v>
@@ -945,10 +965,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>17.10919901199205</v>
+        <v>17.11334091060295</v>
       </c>
       <c r="F7" t="n">
-        <v>16.69011077095796</v>
+        <v>16.67975341968147</v>
       </c>
       <c r="G7" t="n">
         <v>0.2064471879286694</v>
@@ -962,47 +982,50 @@
         </is>
       </c>
       <c r="J7" t="n">
-        <v>61.97794527124018</v>
+        <v>61.96294490592483</v>
       </c>
       <c r="K7" t="n">
-        <v>18.82011891319126</v>
+        <v>18.82467500166324</v>
       </c>
       <c r="L7" t="n">
-        <v>16.25373906139245</v>
+        <v>16.2576738650728</v>
       </c>
       <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr">
+      <c r="N7" t="n">
+        <v>17.79</v>
+      </c>
+      <c r="O7" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P7" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q7" t="n">
+      <c r="R7" t="n">
         <v>1326700000</v>
       </c>
-      <c r="R7" t="inlineStr">
+      <c r="S7" t="inlineStr">
         <is>
           <t>Communication Services</t>
         </is>
       </c>
-      <c r="S7" t="n">
+      <c r="T7" t="n">
         <v>118630000</v>
       </c>
-      <c r="T7" t="inlineStr">
+      <c r="U7" t="inlineStr">
         <is>
           <t>1326.7M</t>
         </is>
       </c>
-      <c r="U7" t="inlineStr">
+      <c r="V7" t="inlineStr">
         <is>
           <t>118.63M</t>
         </is>
@@ -1024,10 +1047,10 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>0.1372375335904927</v>
+        <v>0.1372439192843586</v>
       </c>
       <c r="F8" t="n">
-        <v>73.97247859922771</v>
+        <v>73.88126694342539</v>
       </c>
       <c r="G8" t="n">
         <v>0.2703389830508476</v>
@@ -1041,47 +1064,50 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>7726.698172557801</v>
+        <v>7726.338664250393</v>
       </c>
       <c r="K8" t="n">
-        <v>0.150961286949542</v>
+        <v>0.1509683112127945</v>
       </c>
       <c r="L8" t="n">
-        <v>0.1303756569109681</v>
+        <v>0.1303817233201407</v>
       </c>
       <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr">
+      <c r="N8" t="n">
+        <v>0.1499</v>
+      </c>
+      <c r="O8" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P8" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q8" t="n">
+      <c r="R8" t="n">
         <v>14860000</v>
       </c>
-      <c r="R8" t="inlineStr">
+      <c r="S8" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="S8" t="n">
+      <c r="T8" t="n">
         <v>66390000</v>
       </c>
-      <c r="T8" t="inlineStr">
+      <c r="U8" t="inlineStr">
         <is>
           <t>14.86M</t>
         </is>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="V8" t="inlineStr">
         <is>
           <t>66.39M</t>
         </is>
@@ -1089,7 +1115,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
@@ -1103,10 +1129,10 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>4.359477728624053</v>
+        <v>4.357892197661021</v>
       </c>
       <c r="F9" t="n">
-        <v>7.311694289548949</v>
+        <v>7.290263288531771</v>
       </c>
       <c r="G9" t="n">
         <v>0.05966587112171837</v>
@@ -1120,47 +1146,50 @@
         </is>
       </c>
       <c r="J9" t="n">
-        <v>243.2385404878954</v>
+        <v>243.3270379127636</v>
       </c>
       <c r="K9" t="n">
-        <v>4.795425501486458</v>
+        <v>4.793681417427123</v>
       </c>
       <c r="L9" t="n">
-        <v>4.14150384219285</v>
+        <v>4.13999758777797</v>
       </c>
       <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr">
+      <c r="N9" t="n">
+        <v>4.44</v>
+      </c>
+      <c r="O9" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P9" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q9" t="n">
+      <c r="R9" t="n">
         <v>15962830000</v>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="S9" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="S9" t="n">
+      <c r="T9" t="n">
         <v>2298230000</v>
       </c>
-      <c r="T9" t="inlineStr">
+      <c r="U9" t="inlineStr">
         <is>
           <t>15962.83M</t>
         </is>
       </c>
-      <c r="U9" t="inlineStr">
+      <c r="V9" t="inlineStr">
         <is>
           <t>2298.23M</t>
         </is>
@@ -1208,38 +1237,41 @@
         <v>27.19758381054062</v>
       </c>
       <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr">
+      <c r="N10" t="n">
+        <v>29.57</v>
+      </c>
+      <c r="O10" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P10" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q10" t="n">
+      <c r="R10" t="n">
         <v>1641270000</v>
       </c>
-      <c r="R10" t="inlineStr">
+      <c r="S10" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="S10" t="n">
+      <c r="T10" t="n">
         <v>64540000.00000001</v>
       </c>
-      <c r="T10" t="inlineStr">
+      <c r="U10" t="inlineStr">
         <is>
           <t>1641.27M</t>
         </is>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="V10" t="inlineStr">
         <is>
           <t>64.54M</t>
         </is>
@@ -1247,7 +1279,7 @@
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B11" t="n">
         <v>0</v>
@@ -1261,10 +1293,10 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>13.39339487045958</v>
+        <v>13.39414982586622</v>
       </c>
       <c r="F11" t="n">
-        <v>9.450947786571506</v>
+        <v>9.440241204648455</v>
       </c>
       <c r="G11" t="n">
         <v>0.1198120595144872</v>
@@ -1278,47 +1310,50 @@
         </is>
       </c>
       <c r="J11" t="n">
-        <v>79.17283185152699</v>
+        <v>79.16836930942894</v>
       </c>
       <c r="K11" t="n">
-        <v>14.73273435750553</v>
+        <v>14.73356480845284</v>
       </c>
       <c r="L11" t="n">
-        <v>12.7237251269366</v>
+        <v>12.72444233457291</v>
       </c>
       <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr">
+      <c r="N11" t="n">
+        <v>14.3</v>
+      </c>
+      <c r="O11" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P11" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q11" t="n">
+      <c r="R11" t="n">
         <v>1832710000</v>
       </c>
-      <c r="R11" t="inlineStr">
+      <c r="S11" t="inlineStr">
         <is>
           <t>Industrials</t>
         </is>
       </c>
-      <c r="S11" t="n">
+      <c r="T11" t="n">
         <v>140000000</v>
       </c>
-      <c r="T11" t="inlineStr">
+      <c r="U11" t="inlineStr">
         <is>
           <t>1832.71M</t>
         </is>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="V11" t="inlineStr">
         <is>
           <t>140.0M</t>
         </is>
@@ -1340,10 +1375,10 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>16.61973530437903</v>
+        <v>16.61907448340724</v>
       </c>
       <c r="F12" t="n">
-        <v>7.649896903399812</v>
+        <v>7.642631386133204</v>
       </c>
       <c r="G12" t="n">
         <v>0.0854430379746834</v>
@@ -1357,47 +1392,50 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>63.8032423850098</v>
+        <v>63.80577938071787</v>
       </c>
       <c r="K12" t="n">
-        <v>18.28170883481694</v>
+        <v>18.28098193174796</v>
       </c>
       <c r="L12" t="n">
-        <v>15.78874853916008</v>
+        <v>15.78812075923688</v>
       </c>
       <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr">
+      <c r="N12" t="n">
+        <v>17.15</v>
+      </c>
+      <c r="O12" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P12" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q12" t="n">
+      <c r="R12" t="n">
         <v>2099660000</v>
       </c>
-      <c r="R12" t="inlineStr">
+      <c r="S12" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="S12" t="n">
+      <c r="T12" t="n">
         <v>99790000</v>
       </c>
-      <c r="T12" t="inlineStr">
+      <c r="U12" t="inlineStr">
         <is>
           <t>2099.66M</t>
         </is>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="V12" t="inlineStr">
         <is>
           <t>99.79M</t>
         </is>
@@ -1405,7 +1443,7 @@
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B13" t="n">
         <v>0</v>
@@ -1419,10 +1457,10 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>9.697560983953515</v>
+        <v>9.699095850506463</v>
       </c>
       <c r="F13" t="n">
-        <v>6.757088990325565</v>
+        <v>6.921872631910699</v>
       </c>
       <c r="G13" t="n">
         <v>0.1155334438916528</v>
@@ -1436,47 +1474,50 @@
         </is>
       </c>
       <c r="J13" t="n">
-        <v>109.3463605699025</v>
+        <v>109.3290566815699</v>
       </c>
       <c r="K13" t="n">
-        <v>10.66731708234887</v>
+        <v>10.66900543555711</v>
       </c>
       <c r="L13" t="n">
-        <v>9.21268293475584</v>
+        <v>9.21414105798114</v>
       </c>
       <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr">
+      <c r="N13" t="n">
+        <v>10.09</v>
+      </c>
+      <c r="O13" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P13" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q13" t="n">
+      <c r="R13" t="n">
         <v>2242670000</v>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="S13" t="inlineStr">
         <is>
           <t>Utilities</t>
         </is>
       </c>
-      <c r="S13" t="n">
+      <c r="T13" t="n">
         <v>134690000</v>
       </c>
-      <c r="T13" t="inlineStr">
+      <c r="U13" t="inlineStr">
         <is>
           <t>2242.67M</t>
         </is>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="V13" t="inlineStr">
         <is>
           <t>134.69M</t>
         </is>
@@ -1484,7 +1525,7 @@
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B14" t="n">
         <v>0</v>
@@ -1498,16 +1539,16 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>23.92829309477636</v>
+        <v>23.90999572143198</v>
       </c>
       <c r="F14" t="n">
-        <v>14.46550942781825</v>
+        <v>15.9276544203006</v>
       </c>
       <c r="G14" t="n">
         <v>0.1022880215343204</v>
       </c>
       <c r="H14" t="n">
-        <v>23.5</v>
+        <v>23.66</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1515,47 +1556,50 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>44.31544681436085</v>
+        <v>44.34935967175876</v>
       </c>
       <c r="K14" t="n">
-        <v>26.321122404254</v>
+        <v>26.30099529357518</v>
       </c>
       <c r="L14" t="n">
-        <v>22.73187844003755</v>
+        <v>22.71449593536038</v>
       </c>
       <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr">
+      <c r="N14" t="n">
+        <v>24.57</v>
+      </c>
+      <c r="O14" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O14" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P14" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q14" t="n">
+      <c r="R14" t="n">
         <v>23726730000</v>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="S14" t="inlineStr">
         <is>
           <t>Real Estate</t>
         </is>
       </c>
-      <c r="S14" t="n">
+      <c r="T14" t="n">
         <v>1148010000</v>
       </c>
-      <c r="T14" t="inlineStr">
+      <c r="U14" t="inlineStr">
         <is>
           <t>23726.73M</t>
         </is>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="V14" t="inlineStr">
         <is>
           <t>1148.01M</t>
         </is>
@@ -1563,7 +1607,7 @@
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B15" t="n">
         <v>0</v>
@@ -1573,20 +1617,20 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>LSPD</t>
+          <t>IBRX</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>17.3416324485048</v>
+        <v>5.449205102129668</v>
       </c>
       <c r="F15" t="n">
-        <v>9.385003047810644</v>
+        <v>5.141000751151827</v>
       </c>
       <c r="G15" t="n">
-        <v>0.139135959339263</v>
+        <v>0.05164319248826281</v>
       </c>
       <c r="H15" t="n">
-        <v>16.952209</v>
+        <v>5.2136</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1594,55 +1638,58 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>61.14724223044107</v>
+        <v>194.5959052973755</v>
       </c>
       <c r="K15" t="n">
-        <v>19.07579569335529</v>
+        <v>5.994125612342636</v>
       </c>
       <c r="L15" t="n">
-        <v>16.47455082607956</v>
+        <v>5.176744847023185</v>
       </c>
       <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr">
+      <c r="N15" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="O15" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P15" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q15" t="n">
-        <v>2389310000</v>
-      </c>
-      <c r="R15" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="S15" t="n">
-        <v>136360000</v>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>2389.31M</t>
-        </is>
+      <c r="R15" t="n">
+        <v>2472680000</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>159510000</v>
       </c>
       <c r="U15" t="inlineStr">
         <is>
-          <t>136.36M</t>
+          <t>2472.68M</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>159.51M</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B16" t="n">
         <v>0</v>
@@ -1652,20 +1699,20 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>HBI</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>5.44848371282644</v>
+        <v>8.266060268119839</v>
       </c>
       <c r="F16" t="n">
-        <v>5.139949466920503</v>
+        <v>11.07255944476277</v>
       </c>
       <c r="G16" t="n">
-        <v>0.05164319248826281</v>
+        <v>0.220196353436185</v>
       </c>
       <c r="H16" t="n">
-        <v>5.2136</v>
+        <v>8.15</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1673,55 +1720,58 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>194.6216701545233</v>
+        <v>128.2827569125857</v>
       </c>
       <c r="K16" t="n">
-        <v>5.993332084109084</v>
+        <v>9.092666294931822</v>
       </c>
       <c r="L16" t="n">
-        <v>5.176059527185118</v>
+        <v>7.852757254713847</v>
       </c>
       <c r="M16" t="inlineStr"/>
-      <c r="N16" t="inlineStr">
+      <c r="N16" t="n">
+        <v>8.699999999999999</v>
+      </c>
+      <c r="O16" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P16" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q16" t="n">
-        <v>2472680000</v>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="S16" t="n">
-        <v>159510000</v>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>2472.68M</t>
-        </is>
+      <c r="R16" t="n">
+        <v>2525130000</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>347400000</v>
       </c>
       <c r="U16" t="inlineStr">
         <is>
-          <t>159.51M</t>
+          <t>2525.13M</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>347.4M</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="B17" t="n">
         <v>0</v>
@@ -1731,20 +1781,20 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>HBI</t>
+          <t>VCYT</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>8.271337784696621</v>
+        <v>39.26629619620718</v>
       </c>
       <c r="F17" t="n">
-        <v>11.03592787674254</v>
+        <v>11.06094029372027</v>
       </c>
       <c r="G17" t="n">
-        <v>0.220196353436185</v>
+        <v>0.1485999445522595</v>
       </c>
       <c r="H17" t="n">
-        <v>8.15</v>
+        <v>37.38</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1752,55 +1802,58 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>128.2009062623349</v>
+        <v>27.00516989688541</v>
       </c>
       <c r="K17" t="n">
-        <v>9.098471563166283</v>
+        <v>43.1929258158279</v>
       </c>
       <c r="L17" t="n">
-        <v>7.85777089546179</v>
+        <v>37.30298138639682</v>
       </c>
       <c r="M17" t="inlineStr"/>
-      <c r="N17" t="inlineStr">
+      <c r="N17" t="n">
+        <v>41.43</v>
+      </c>
+      <c r="O17" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O17" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P17" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q17" t="n">
-        <v>2525130000</v>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="S17" t="n">
-        <v>347400000</v>
-      </c>
-      <c r="T17" t="inlineStr">
-        <is>
-          <t>2525.13M</t>
-        </is>
+      <c r="R17" t="n">
+        <v>2543950000</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>75650000</v>
       </c>
       <c r="U17" t="inlineStr">
         <is>
-          <t>347.4M</t>
+          <t>2543.95M</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>75.65M</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="B18" t="n">
         <v>0</v>
@@ -1810,20 +1863,20 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>VCYT</t>
+          <t>IHRT</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>39.26629897023958</v>
+        <v>2.459132788978218</v>
       </c>
       <c r="F18" t="n">
-        <v>11.06368672100913</v>
+        <v>54.25699679526715</v>
       </c>
       <c r="G18" t="n">
-        <v>0.1485999445522595</v>
+        <v>0.5734072022160664</v>
       </c>
       <c r="H18" t="n">
-        <v>37.38</v>
+        <v>2.15</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1831,49 +1884,52 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>27.00516798906067</v>
+        <v>431.2060758787241</v>
       </c>
       <c r="K18" t="n">
-        <v>43.19292886726354</v>
+        <v>2.70504606787604</v>
       </c>
       <c r="L18" t="n">
-        <v>37.3029840217276</v>
+        <v>2.336176149529307</v>
       </c>
       <c r="M18" t="inlineStr"/>
-      <c r="N18" t="inlineStr">
+      <c r="N18" t="n">
+        <v>2.84</v>
+      </c>
+      <c r="O18" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P18" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q18" t="n">
-        <v>2543950000</v>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="S18" t="n">
-        <v>75650000</v>
-      </c>
-      <c r="T18" t="inlineStr">
-        <is>
-          <t>2543.95M</t>
-        </is>
+      <c r="R18" t="n">
+        <v>256920000</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="T18" t="n">
+        <v>116040000</v>
       </c>
       <c r="U18" t="inlineStr">
         <is>
-          <t>75.65M</t>
+          <t>256.92M</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>116.04M</t>
         </is>
       </c>
     </row>
@@ -1889,20 +1945,20 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>IHRT</t>
+          <t>GH</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2.458667222957222</v>
+        <v>30.58852292504103</v>
       </c>
       <c r="F19" t="n">
-        <v>54.38631211483916</v>
+        <v>14.27817040377623</v>
       </c>
       <c r="G19" t="n">
-        <v>0.5734072022160664</v>
+        <v>0.3897087378640778</v>
       </c>
       <c r="H19" t="n">
-        <v>2.15</v>
+        <v>28.59</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1910,55 +1966,58 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>431.2877277977402</v>
+        <v>34.66636825186216</v>
       </c>
       <c r="K19" t="n">
-        <v>2.704533945252944</v>
+        <v>33.64737521754513</v>
       </c>
       <c r="L19" t="n">
-        <v>2.335733861809361</v>
+        <v>29.05909677878898</v>
       </c>
       <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr">
+      <c r="N19" t="n">
+        <v>33.6379</v>
+      </c>
+      <c r="O19" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O19" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P19" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q19" t="n">
-        <v>256920000</v>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="S19" t="n">
-        <v>116040000</v>
-      </c>
-      <c r="T19" t="inlineStr">
-        <is>
-          <t>256.92M</t>
-        </is>
+      <c r="R19" t="n">
+        <v>2563740000</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="T19" t="n">
+        <v>117720000</v>
       </c>
       <c r="U19" t="inlineStr">
         <is>
-          <t>116.04M</t>
+          <t>2563.74M</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>117.72M</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B20" t="n">
         <v>0</v>
@@ -1968,76 +2027,79 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>TNXP</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>30.58718493103747</v>
+        <v>0.1410002690423899</v>
       </c>
       <c r="F20" t="n">
-        <v>14.35672150347875</v>
+        <v>5.992068315644742</v>
       </c>
       <c r="G20" t="n">
-        <v>0.3897087378640778</v>
+        <v>0.07758620689655175</v>
       </c>
       <c r="H20" t="n">
-        <v>28.59</v>
+        <v>0.139</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>09:30:00</t>
+          <t>10:30:00</t>
         </is>
       </c>
       <c r="J20" t="n">
-        <v>34.66788468408534</v>
+        <v>7520.503380608489</v>
       </c>
       <c r="K20" t="n">
-        <v>33.64590342414122</v>
+        <v>0.1551002959466289</v>
       </c>
       <c r="L20" t="n">
-        <v>29.0578256844856</v>
+        <v>0.1339502555902704</v>
       </c>
       <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr">
+      <c r="N20" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P20" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q20" t="n">
-        <v>2563740000</v>
-      </c>
-      <c r="R20" t="inlineStr">
+      <c r="R20" t="n">
+        <v>26070000</v>
+      </c>
+      <c r="S20" t="inlineStr">
         <is>
           <t>Healthcare</t>
         </is>
       </c>
-      <c r="S20" t="n">
-        <v>117720000</v>
-      </c>
-      <c r="T20" t="inlineStr">
-        <is>
-          <t>2563.74M</t>
-        </is>
+      <c r="T20" t="n">
+        <v>137260000</v>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>117.72M</t>
+          <t>26.07M</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>137.26M</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B21" t="n">
         <v>0</v>
@@ -2047,76 +2109,79 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>TNXP</t>
+          <t>CAN</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>0.1409947177045335</v>
+        <v>1.415842377925173</v>
       </c>
       <c r="F21" t="n">
-        <v>5.707379511136475</v>
+        <v>5.797106239303663</v>
       </c>
       <c r="G21" t="n">
-        <v>0.07758620689655175</v>
+        <v>0.07270072992700723</v>
       </c>
       <c r="H21" t="n">
-        <v>0.139</v>
+        <v>1.4103</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>10:30:00</t>
+          <t>09:30:00</t>
         </is>
       </c>
       <c r="J21" t="n">
-        <v>7520.799482872433</v>
+        <v>748.9484822130687</v>
       </c>
       <c r="K21" t="n">
-        <v>0.1550941894749868</v>
+        <v>1.55742661571769</v>
       </c>
       <c r="L21" t="n">
-        <v>0.1339449818193068</v>
+        <v>1.345050259028914</v>
       </c>
       <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr">
+      <c r="N21" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="O21" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P21" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q21" t="n">
-        <v>26070000</v>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="S21" t="n">
-        <v>137260000</v>
-      </c>
-      <c r="T21" t="inlineStr">
-        <is>
-          <t>26.07M</t>
-        </is>
+      <c r="R21" t="n">
+        <v>264260000</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="T21" t="n">
+        <v>149260000</v>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>137.26M</t>
+          <t>264.26M</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>149.26M</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
-        <v>27</v>
+        <v>9</v>
       </c>
       <c r="B22" t="n">
         <v>0</v>
@@ -2126,76 +2191,79 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>CAN</t>
+          <t>BNGO</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1.415599867321131</v>
+        <v>0.3020659672464759</v>
       </c>
       <c r="F22" t="n">
-        <v>5.854230455117648</v>
+        <v>13.16960601378603</v>
       </c>
       <c r="G22" t="n">
-        <v>0.07270072992700723</v>
+        <v>0.1086694548805558</v>
       </c>
       <c r="H22" t="n">
-        <v>1.4103</v>
+        <v>0.3005</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>09:30:00</t>
+          <t>10:00:00</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>749.0767867947591</v>
+        <v>3510.468291632318</v>
       </c>
       <c r="K22" t="n">
-        <v>1.557159854053244</v>
+        <v>0.3322725639711235</v>
       </c>
       <c r="L22" t="n">
-        <v>1.344819873955075</v>
+        <v>0.2869626688841521</v>
       </c>
       <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr">
+      <c r="N22" t="n">
+        <v>0.3128</v>
+      </c>
+      <c r="O22" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P22" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q22" t="n">
-        <v>264260000</v>
-      </c>
-      <c r="R22" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="S22" t="n">
-        <v>149260000</v>
-      </c>
-      <c r="T22" t="inlineStr">
-        <is>
-          <t>264.26M</t>
-        </is>
+      <c r="R22" t="n">
+        <v>27560000</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="T22" t="n">
+        <v>85450000</v>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>149.26M</t>
+          <t>27.56M</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>85.45M</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="1" t="n">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="B23" t="n">
         <v>0</v>
@@ -2205,20 +2273,20 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>BRY</t>
         </is>
       </c>
       <c r="E23" t="n">
-        <v>8.106445224073747</v>
+        <v>5.554250071247506</v>
       </c>
       <c r="F23" t="n">
-        <v>24.65031608371826</v>
+        <v>6.348682527004418</v>
       </c>
       <c r="G23" t="n">
-        <v>0.2442196531791907</v>
+        <v>0.0554561717352416</v>
       </c>
       <c r="H23" t="n">
-        <v>7.68</v>
+        <v>5.1</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -2226,55 +2294,58 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>130.8086307486475</v>
+        <v>190.9156027182319</v>
       </c>
       <c r="K23" t="n">
-        <v>8.917089746481121</v>
+        <v>6.109675078372257</v>
       </c>
       <c r="L23" t="n">
-        <v>7.70112296287006</v>
+        <v>5.276537567685131</v>
       </c>
       <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr">
+      <c r="N23" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="O23" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O23" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P23" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q23" t="n">
-        <v>2693640000</v>
-      </c>
-      <c r="R23" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="S23" t="n">
-        <v>110970000</v>
-      </c>
-      <c r="T23" t="inlineStr">
-        <is>
-          <t>2693.64M</t>
-        </is>
+      <c r="R23" t="n">
+        <v>401630000</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="T23" t="n">
+        <v>74970000</v>
       </c>
       <c r="U23" t="inlineStr">
         <is>
-          <t>110.97M</t>
+          <t>401.63M</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>74.97M</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="1" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="B24" t="n">
         <v>0</v>
@@ -2284,76 +2355,79 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>BNGO</t>
+          <t>VRT</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>0.3019806773693406</v>
+        <v>123.4008171684077</v>
       </c>
       <c r="F24" t="n">
-        <v>12.77660683123642</v>
+        <v>5.8167452440548</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1086694548805558</v>
+        <v>0.06916080315771399</v>
       </c>
       <c r="H24" t="n">
-        <v>0.3005</v>
+        <v>122</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>09:30:00</t>
         </is>
       </c>
       <c r="J24" t="n">
-        <v>3511.459770331846</v>
+        <v>8.593079238307304</v>
       </c>
       <c r="K24" t="n">
-        <v>0.3321787451062747</v>
+        <v>135.7408988852485</v>
       </c>
       <c r="L24" t="n">
-        <v>0.2868816435008736</v>
+        <v>117.2307763099873</v>
       </c>
       <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr">
+      <c r="N24" t="n">
+        <v>124.855</v>
+      </c>
+      <c r="O24" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O24" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P24" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q24" t="n">
-        <v>27560000</v>
-      </c>
-      <c r="R24" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="S24" t="n">
-        <v>85450000</v>
-      </c>
-      <c r="T24" t="inlineStr">
-        <is>
-          <t>27.56M</t>
-        </is>
+      <c r="R24" t="n">
+        <v>42058070000</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="T24" t="n">
+        <v>365720000</v>
       </c>
       <c r="U24" t="inlineStr">
         <is>
-          <t>85.45M</t>
+          <t>42058.07M</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>365.72M</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="B25" t="n">
         <v>0</v>
@@ -2363,76 +2437,79 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>DV</t>
+          <t>VALE</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>19.90976270944414</v>
+        <v>11.21466851788707</v>
       </c>
       <c r="F25" t="n">
-        <v>6.042088857474317</v>
+        <v>16.07368218687569</v>
       </c>
       <c r="G25" t="n">
-        <v>0.08916177255739445</v>
+        <v>0.06197183098591551</v>
       </c>
       <c r="H25" t="n">
-        <v>19.72</v>
+        <v>11.18</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>10:00:00</t>
+          <t>09:30:00</t>
         </is>
       </c>
       <c r="J25" t="n">
-        <v>53.2599516867675</v>
+        <v>94.5541099416986</v>
       </c>
       <c r="K25" t="n">
-        <v>21.90073898038855</v>
+        <v>12.33613536967578</v>
       </c>
       <c r="L25" t="n">
-        <v>18.91427457397193</v>
+        <v>10.65393509199272</v>
       </c>
       <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr">
+      <c r="N25" t="n">
+        <v>11.32</v>
+      </c>
+      <c r="O25" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P25" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q25" t="n">
-        <v>2963800000</v>
-      </c>
-      <c r="R25" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="S25" t="n">
-        <v>142770000</v>
-      </c>
-      <c r="T25" t="inlineStr">
-        <is>
-          <t>2963.8M</t>
-        </is>
+      <c r="R25" t="n">
+        <v>45143520000</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>Basic Materials</t>
+        </is>
+      </c>
+      <c r="T25" t="n">
+        <v>4270860000</v>
       </c>
       <c r="U25" t="inlineStr">
         <is>
-          <t>142.77M</t>
+          <t>45143.52M</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>4270.86M</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="n">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="B26" t="n">
         <v>0</v>
@@ -2442,20 +2519,20 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>TDS</t>
+          <t>GOTU</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>33.86224489035541</v>
+        <v>3.210649624154813</v>
       </c>
       <c r="F26" t="n">
-        <v>12.26277496540251</v>
+        <v>13.94745776538515</v>
       </c>
       <c r="G26" t="n">
-        <v>0.1291850400130655</v>
+        <v>0.08441558441558435</v>
       </c>
       <c r="H26" t="n">
-        <v>32.45</v>
+        <v>3.2101</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2463,55 +2540,58 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>31.31490553663852</v>
+        <v>330.2736592689222</v>
       </c>
       <c r="K26" t="n">
-        <v>37.24846937939095</v>
+        <v>3.531714586570295</v>
       </c>
       <c r="L26" t="n">
-        <v>32.16913264583764</v>
+        <v>3.050117142947073</v>
       </c>
       <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr">
+      <c r="N26" t="n">
+        <v>3.34</v>
+      </c>
+      <c r="O26" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O26" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P26" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q26" t="n">
-        <v>3199030000</v>
-      </c>
-      <c r="R26" t="inlineStr">
-        <is>
-          <t>Communication Services</t>
-        </is>
-      </c>
-      <c r="S26" t="n">
-        <v>98280000</v>
-      </c>
-      <c r="T26" t="inlineStr">
-        <is>
-          <t>3199.03M</t>
-        </is>
+      <c r="R26" t="n">
+        <v>469260000</v>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>Consumer Defensive</t>
+        </is>
+      </c>
+      <c r="T26" t="n">
+        <v>148410000</v>
       </c>
       <c r="U26" t="inlineStr">
         <is>
-          <t>98.28M</t>
+          <t>469.26M</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>148.41M</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="1" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="B27" t="n">
         <v>0</v>
@@ -2521,20 +2601,20 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>BRY</t>
+          <t>DNMR</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>5.553926078520326</v>
+        <v>0.3242314875110855</v>
       </c>
       <c r="F27" t="n">
-        <v>6.381652503638898</v>
+        <v>5.881203028493514</v>
       </c>
       <c r="G27" t="n">
-        <v>0.0554561717352416</v>
+        <v>0.1298701298701298</v>
       </c>
       <c r="H27" t="n">
-        <v>5.1</v>
+        <v>0.3196</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2542,55 +2622,58 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>190.9267399328637</v>
+        <v>3270.481248258608</v>
       </c>
       <c r="K27" t="n">
-        <v>6.109318686372358</v>
+        <v>0.3566546362621941</v>
       </c>
       <c r="L27" t="n">
-        <v>5.276229774594309</v>
+        <v>0.3080199131355312</v>
       </c>
       <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr">
+      <c r="N27" t="n">
+        <v>0.348</v>
+      </c>
+      <c r="O27" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O27" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P27" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q27" t="n">
-        <v>401630000</v>
-      </c>
-      <c r="R27" t="inlineStr">
-        <is>
-          <t>Energy</t>
-        </is>
-      </c>
-      <c r="S27" t="n">
-        <v>74970000</v>
-      </c>
-      <c r="T27" t="inlineStr">
-        <is>
-          <t>401.63M</t>
-        </is>
+      <c r="R27" t="n">
+        <v>49110000</v>
+      </c>
+      <c r="S27" t="inlineStr">
+        <is>
+          <t>Basic Materials</t>
+        </is>
+      </c>
+      <c r="T27" t="n">
+        <v>108900000</v>
       </c>
       <c r="U27" t="inlineStr">
         <is>
-          <t>74.97M</t>
+          <t>49.11M</t>
+        </is>
+      </c>
+      <c r="V27" t="inlineStr">
+        <is>
+          <t>108.9M</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="1" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
       <c r="B28" t="n">
         <v>0</v>
@@ -2600,20 +2683,20 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>VRT</t>
+          <t>ALT</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>123.0144433739607</v>
+        <v>7.828426404464473</v>
       </c>
       <c r="F28" t="n">
-        <v>5.469741588646422</v>
+        <v>13.67959908028419</v>
       </c>
       <c r="G28" t="n">
-        <v>0.06916080315771399</v>
+        <v>0.127450980392157</v>
       </c>
       <c r="H28" t="n">
-        <v>122</v>
+        <v>7.4599</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -2621,55 +2704,58 @@
         </is>
       </c>
       <c r="J28" t="n">
-        <v>8.620069082265671</v>
+        <v>135.4541698693455</v>
       </c>
       <c r="K28" t="n">
-        <v>135.3158877113568</v>
+        <v>8.611269044910919</v>
       </c>
       <c r="L28" t="n">
-        <v>116.8637212052627</v>
+        <v>7.43700508424125</v>
       </c>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr">
+      <c r="N28" t="n">
+        <v>8.050000000000001</v>
+      </c>
+      <c r="O28" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O28" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P28" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q28" t="n">
-        <v>42058070000</v>
-      </c>
-      <c r="R28" t="inlineStr">
-        <is>
-          <t>Industrials</t>
-        </is>
-      </c>
-      <c r="S28" t="n">
-        <v>365720000</v>
-      </c>
-      <c r="T28" t="inlineStr">
-        <is>
-          <t>42058.07M</t>
-        </is>
+      <c r="R28" t="n">
+        <v>490380000</v>
+      </c>
+      <c r="S28" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="T28" t="n">
+        <v>70480000</v>
       </c>
       <c r="U28" t="inlineStr">
         <is>
-          <t>365.72M</t>
+          <t>490.38M</t>
+        </is>
+      </c>
+      <c r="V28" t="inlineStr">
+        <is>
+          <t>70.48M</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="1" t="n">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="B29" t="n">
         <v>0</v>
@@ -2679,20 +2765,20 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>VALE</t>
+          <t>CPRI</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>11.21588472719695</v>
+        <v>22.41304877366974</v>
       </c>
       <c r="F29" t="n">
-        <v>15.12736458563343</v>
+        <v>7.064314252393315</v>
       </c>
       <c r="G29" t="n">
-        <v>0.06197183098591551</v>
+        <v>0.07109227871939744</v>
       </c>
       <c r="H29" t="n">
-        <v>11.18</v>
+        <v>20.63</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -2700,55 +2786,58 @@
         </is>
       </c>
       <c r="J29" t="n">
-        <v>94.5438568416003</v>
+        <v>47.31141268231753</v>
       </c>
       <c r="K29" t="n">
-        <v>12.33747319991665</v>
+        <v>24.65435365103672</v>
       </c>
       <c r="L29" t="n">
-        <v>10.65509049083711</v>
+        <v>21.29239633498626</v>
       </c>
       <c r="M29" t="inlineStr"/>
-      <c r="N29" t="inlineStr">
+      <c r="N29" t="n">
+        <v>22.8491</v>
+      </c>
+      <c r="O29" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O29" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P29" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q29" t="n">
-        <v>45143520000</v>
-      </c>
-      <c r="R29" t="inlineStr">
-        <is>
-          <t>Basic Materials</t>
-        </is>
-      </c>
-      <c r="S29" t="n">
-        <v>4270860000</v>
-      </c>
-      <c r="T29" t="inlineStr">
-        <is>
-          <t>45143.52M</t>
-        </is>
+      <c r="R29" t="n">
+        <v>4951890000</v>
+      </c>
+      <c r="S29" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="T29" t="n">
+        <v>115100000</v>
       </c>
       <c r="U29" t="inlineStr">
         <is>
-          <t>4270.86M</t>
+          <t>4951.89M</t>
+        </is>
+      </c>
+      <c r="V29" t="inlineStr">
+        <is>
+          <t>115.1M</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>26</v>
+        <v>4</v>
       </c>
       <c r="B30" t="n">
         <v>0</v>
@@ -2758,20 +2847,20 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>GOTU</t>
+          <t>MC</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>3.21260947895908</v>
+        <v>80.83316346536778</v>
       </c>
       <c r="F30" t="n">
-        <v>13.51795028029544</v>
+        <v>6.613627607728315</v>
       </c>
       <c r="G30" t="n">
-        <v>0.08441558441558435</v>
+        <v>0.05810179174240469</v>
       </c>
       <c r="H30" t="n">
-        <v>3.2101</v>
+        <v>77</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2779,55 +2868,58 @@
         </is>
       </c>
       <c r="J30" t="n">
-        <v>330.0721755772129</v>
+        <v>13.1182914850823</v>
       </c>
       <c r="K30" t="n">
-        <v>3.533870426854989</v>
+        <v>88.91647981190455</v>
       </c>
       <c r="L30" t="n">
-        <v>3.051979005011126</v>
+        <v>76.79150529209939</v>
       </c>
       <c r="M30" t="inlineStr"/>
-      <c r="N30" t="inlineStr">
+      <c r="N30" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="O30" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O30" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P30" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q30" t="n">
-        <v>469260000</v>
-      </c>
-      <c r="R30" t="inlineStr">
-        <is>
-          <t>Consumer Defensive</t>
-        </is>
-      </c>
-      <c r="S30" t="n">
-        <v>148410000</v>
-      </c>
-      <c r="T30" t="inlineStr">
-        <is>
-          <t>469.26M</t>
-        </is>
+      <c r="R30" t="n">
+        <v>4970230000</v>
+      </c>
+      <c r="S30" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="T30" t="n">
+        <v>70120000</v>
       </c>
       <c r="U30" t="inlineStr">
         <is>
-          <t>148.41M</t>
+          <t>4970.23M</t>
+        </is>
+      </c>
+      <c r="V30" t="inlineStr">
+        <is>
+          <t>70.12M</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="B31" t="n">
         <v>0</v>
@@ -2837,20 +2929,20 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>DNMR</t>
+          <t>EBS</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>0.3244655543351159</v>
+        <v>11.9360979744265</v>
       </c>
       <c r="F31" t="n">
-        <v>5.806244595763078</v>
+        <v>28.34709929907042</v>
       </c>
       <c r="G31" t="n">
-        <v>0.1298701298701298</v>
+        <v>0.3882224645583425</v>
       </c>
       <c r="H31" t="n">
-        <v>0.3196</v>
+        <v>10.9001</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
@@ -2858,55 +2950,58 @@
         </is>
       </c>
       <c r="J31" t="n">
-        <v>3268.121949563868</v>
+        <v>88.83916689289318</v>
       </c>
       <c r="K31" t="n">
-        <v>0.3569121097686275</v>
+        <v>13.12970777186915</v>
       </c>
       <c r="L31" t="n">
-        <v>0.3082422766183601</v>
+        <v>11.33929307570518</v>
       </c>
       <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr">
+      <c r="N31" t="n">
+        <v>12.73</v>
+      </c>
+      <c r="O31" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O31" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P31" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q31" t="n">
-        <v>49110000</v>
-      </c>
-      <c r="R31" t="inlineStr">
-        <is>
-          <t>Basic Materials</t>
-        </is>
-      </c>
-      <c r="S31" t="n">
-        <v>108900000</v>
-      </c>
-      <c r="T31" t="inlineStr">
-        <is>
-          <t>49.11M</t>
-        </is>
+      <c r="R31" t="n">
+        <v>549920000</v>
+      </c>
+      <c r="S31" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="T31" t="n">
+        <v>51910000</v>
       </c>
       <c r="U31" t="inlineStr">
         <is>
-          <t>108.9M</t>
+          <t>549.92M</t>
+        </is>
+      </c>
+      <c r="V31" t="inlineStr">
+        <is>
+          <t>51.91M</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="B32" t="n">
         <v>0</v>
@@ -2916,20 +3011,20 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>ALT</t>
+          <t>LAAC</t>
         </is>
       </c>
       <c r="E32" t="n">
-        <v>7.82511144184494</v>
+        <v>3.381182329995576</v>
       </c>
       <c r="F32" t="n">
-        <v>13.53622481955971</v>
+        <v>5.121877793081503</v>
       </c>
       <c r="G32" t="n">
-        <v>0.127450980392157</v>
+        <v>0.09119496855345913</v>
       </c>
       <c r="H32" t="n">
-        <v>7.4599</v>
+        <v>3.28</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
@@ -2937,55 +3032,58 @@
         </is>
       </c>
       <c r="J32" t="n">
-        <v>135.5115525038439</v>
+        <v>313.6160361992036</v>
       </c>
       <c r="K32" t="n">
-        <v>8.607622586029434</v>
+        <v>3.719300562995134</v>
       </c>
       <c r="L32" t="n">
-        <v>7.433855869752692</v>
+        <v>3.212123213495797</v>
       </c>
       <c r="M32" t="inlineStr"/>
-      <c r="N32" t="inlineStr">
+      <c r="N32" t="n">
+        <v>3.47</v>
+      </c>
+      <c r="O32" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O32" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P32" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q32" t="n">
-        <v>490380000</v>
-      </c>
-      <c r="R32" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="S32" t="n">
-        <v>70480000</v>
-      </c>
-      <c r="T32" t="inlineStr">
-        <is>
-          <t>490.38M</t>
-        </is>
+      <c r="R32" t="n">
+        <v>558100000</v>
+      </c>
+      <c r="S32" t="inlineStr">
+        <is>
+          <t>Basic Materials</t>
+        </is>
+      </c>
+      <c r="T32" t="n">
+        <v>136320000</v>
       </c>
       <c r="U32" t="inlineStr">
         <is>
-          <t>70.48M</t>
+          <t>558.1M</t>
+        </is>
+      </c>
+      <c r="V32" t="inlineStr">
+        <is>
+          <t>136.32M</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="1" t="n">
-        <v>15</v>
+        <v>28</v>
       </c>
       <c r="B33" t="n">
         <v>0</v>
@@ -2995,20 +3093,20 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CPRI</t>
+          <t>LYFT</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>22.41330518393556</v>
+        <v>18.17786074440388</v>
       </c>
       <c r="F33" t="n">
-        <v>6.599195749835499</v>
+        <v>29.25727117245391</v>
       </c>
       <c r="G33" t="n">
-        <v>0.07109227871939744</v>
+        <v>0.3418894830659536</v>
       </c>
       <c r="H33" t="n">
-        <v>20.63</v>
+        <v>17.8</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -3016,55 +3114,58 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>47.31087143541964</v>
+        <v>58.33431199138467</v>
       </c>
       <c r="K33" t="n">
-        <v>24.65463570232912</v>
+        <v>19.99564681884427</v>
       </c>
       <c r="L33" t="n">
-        <v>21.29263992473879</v>
+        <v>17.26896770718368</v>
       </c>
       <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr">
+      <c r="N33" t="n">
+        <v>18.82</v>
+      </c>
+      <c r="O33" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O33" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P33" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q33" t="n">
-        <v>4951890000</v>
-      </c>
-      <c r="R33" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="S33" t="n">
-        <v>115100000</v>
-      </c>
-      <c r="T33" t="inlineStr">
-        <is>
-          <t>4951.89M</t>
-        </is>
+      <c r="R33" t="n">
+        <v>5758650000</v>
+      </c>
+      <c r="S33" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="T33" t="n">
+        <v>349630000</v>
       </c>
       <c r="U33" t="inlineStr">
         <is>
-          <t>115.1M</t>
+          <t>5758.65M</t>
+        </is>
+      </c>
+      <c r="V33" t="inlineStr">
+        <is>
+          <t>349.63M</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="1" t="n">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="B34" t="n">
         <v>0</v>
@@ -3074,20 +3175,20 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>EBS</t>
+          <t>FCX</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>11.9360979744265</v>
+        <v>48.77630238844687</v>
       </c>
       <c r="F34" t="n">
-        <v>28.34709929907042</v>
+        <v>7.733525537879308</v>
       </c>
       <c r="G34" t="n">
-        <v>0.3882224645583425</v>
+        <v>0.06400000000000002</v>
       </c>
       <c r="H34" t="n">
-        <v>10.9001</v>
+        <v>48.68</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
@@ -3095,55 +3196,58 @@
         </is>
       </c>
       <c r="J34" t="n">
-        <v>88.83916689289318</v>
+        <v>21.73992180783191</v>
       </c>
       <c r="K34" t="n">
-        <v>13.12970777186915</v>
+        <v>53.65393262729156</v>
       </c>
       <c r="L34" t="n">
-        <v>11.33929307570518</v>
+        <v>46.33748726902453</v>
       </c>
       <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr">
+      <c r="N34" t="n">
+        <v>49.21</v>
+      </c>
+      <c r="O34" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O34" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P34" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q34" t="n">
-        <v>549920000</v>
-      </c>
-      <c r="R34" t="inlineStr">
-        <is>
-          <t>Healthcare</t>
-        </is>
-      </c>
-      <c r="S34" t="n">
-        <v>51910000</v>
-      </c>
-      <c r="T34" t="inlineStr">
-        <is>
-          <t>549.92M</t>
-        </is>
+      <c r="R34" t="n">
+        <v>68883070000</v>
+      </c>
+      <c r="S34" t="inlineStr">
+        <is>
+          <t>Basic Materials</t>
+        </is>
+      </c>
+      <c r="T34" t="n">
+        <v>1425790000</v>
       </c>
       <c r="U34" t="inlineStr">
         <is>
-          <t>51.91M</t>
+          <t>68883.07M</t>
+        </is>
+      </c>
+      <c r="V34" t="inlineStr">
+        <is>
+          <t>1425.79M</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="1" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="B35" t="n">
         <v>0</v>
@@ -3153,76 +3257,79 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>LAAC</t>
+          <t>LUXH</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>3.381102129540341</v>
+        <v>0.05461780491246219</v>
       </c>
       <c r="F35" t="n">
-        <v>5.121705721850494</v>
+        <v>8.085129173698059</v>
       </c>
       <c r="G35" t="n">
-        <v>0.09119496855345913</v>
+        <v>0.1976047904191617</v>
       </c>
       <c r="H35" t="n">
-        <v>3.28</v>
+        <v>0.05</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>09:30:00</t>
+          <t>11:00:00</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>313.6234752376912</v>
+        <v>19414.78610682959</v>
       </c>
       <c r="K35" t="n">
-        <v>3.719212342494375</v>
+        <v>0.0600795854037084</v>
       </c>
       <c r="L35" t="n">
-        <v>3.212047023063324</v>
+        <v>0.05188691466683908</v>
       </c>
       <c r="M35" t="inlineStr"/>
-      <c r="N35" t="inlineStr">
+      <c r="N35" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="O35" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O35" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P35" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q35" t="n">
-        <v>558100000</v>
-      </c>
-      <c r="R35" t="inlineStr">
-        <is>
-          <t>Basic Materials</t>
-        </is>
-      </c>
-      <c r="S35" t="n">
-        <v>136320000</v>
-      </c>
-      <c r="T35" t="inlineStr">
-        <is>
-          <t>558.1M</t>
-        </is>
+      <c r="R35" t="n">
+        <v>7110000</v>
+      </c>
+      <c r="S35" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="T35" t="n">
+        <v>99180000</v>
       </c>
       <c r="U35" t="inlineStr">
         <is>
-          <t>136.32M</t>
+          <t>7.11M</t>
+        </is>
+      </c>
+      <c r="V35" t="inlineStr">
+        <is>
+          <t>99.18M</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="B36" t="n">
         <v>0</v>
@@ -3232,20 +3339,20 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>LYFT</t>
+          <t>MTC</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>18.1754738140739</v>
+        <v>0.4078283009466867</v>
       </c>
       <c r="F36" t="n">
-        <v>27.91283713538935</v>
+        <v>23.49735967520067</v>
       </c>
       <c r="G36" t="n">
-        <v>0.3418894830659536</v>
+        <v>0.180327868852459</v>
       </c>
       <c r="H36" t="n">
-        <v>17.8</v>
+        <v>0.3868</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -3253,284 +3360,50 @@
         </is>
       </c>
       <c r="J36" t="n">
-        <v>58.34197286119171</v>
+        <v>2600.096652288532</v>
       </c>
       <c r="K36" t="n">
-        <v>19.99302119548129</v>
+        <v>0.4486111310413553</v>
       </c>
       <c r="L36" t="n">
-        <v>17.26670012337021</v>
+        <v>0.3874368858993523</v>
       </c>
       <c r="M36" t="inlineStr"/>
-      <c r="N36" t="inlineStr">
+      <c r="N36" t="n">
+        <v>0.432</v>
+      </c>
+      <c r="O36" t="inlineStr">
         <is>
           <t>12:30:00</t>
         </is>
       </c>
-      <c r="O36" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
       <c r="P36" t="inlineStr">
         <is>
+          <t>10:30:00</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
           <t>15:30:00</t>
         </is>
       </c>
-      <c r="Q36" t="n">
-        <v>5758650000</v>
-      </c>
-      <c r="R36" t="inlineStr">
+      <c r="R36" t="n">
+        <v>77110000</v>
+      </c>
+      <c r="S36" t="inlineStr">
         <is>
           <t>Technology</t>
         </is>
       </c>
-      <c r="S36" t="n">
-        <v>349630000</v>
-      </c>
-      <c r="T36" t="inlineStr">
-        <is>
-          <t>5758.65M</t>
-        </is>
+      <c r="T36" t="n">
+        <v>198780000</v>
       </c>
       <c r="U36" t="inlineStr">
         <is>
-          <t>349.63M</t>
-        </is>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" s="1" t="n">
-        <v>35</v>
-      </c>
-      <c r="B37" t="n">
-        <v>0</v>
-      </c>
-      <c r="C37" s="2" t="n">
-        <v>45603</v>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>FCX</t>
-        </is>
-      </c>
-      <c r="E37" t="n">
-        <v>48.75719415605986</v>
-      </c>
-      <c r="F37" t="n">
-        <v>7.498708164663928</v>
-      </c>
-      <c r="G37" t="n">
-        <v>0.06400000000000002</v>
-      </c>
-      <c r="H37" t="n">
-        <v>48.58</v>
-      </c>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>09:30:00</t>
-        </is>
-      </c>
-      <c r="J37" t="n">
-        <v>21.748441811601</v>
-      </c>
-      <c r="K37" t="n">
-        <v>53.63291357166585</v>
-      </c>
-      <c r="L37" t="n">
-        <v>46.31933444825687</v>
-      </c>
-      <c r="M37" t="inlineStr"/>
-      <c r="N37" t="inlineStr">
-        <is>
-          <t>12:30:00</t>
-        </is>
-      </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="P37" t="inlineStr">
-        <is>
-          <t>15:30:00</t>
-        </is>
-      </c>
-      <c r="Q37" t="n">
-        <v>68883070000</v>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>Basic Materials</t>
-        </is>
-      </c>
-      <c r="S37" t="n">
-        <v>1425790000</v>
-      </c>
-      <c r="T37" t="inlineStr">
-        <is>
-          <t>68883.07M</t>
-        </is>
-      </c>
-      <c r="U37" t="inlineStr">
-        <is>
-          <t>1425.79M</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="n">
-        <v>11</v>
-      </c>
-      <c r="B38" t="n">
-        <v>0</v>
-      </c>
-      <c r="C38" s="2" t="n">
-        <v>45603</v>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>LUXH</t>
-        </is>
-      </c>
-      <c r="E38" t="n">
-        <v>0.05463719925869764</v>
-      </c>
-      <c r="F38" t="n">
-        <v>7.696495759612235</v>
-      </c>
-      <c r="G38" t="n">
-        <v>0.1976047904191617</v>
-      </c>
-      <c r="H38" t="n">
-        <v>0.05</v>
-      </c>
-      <c r="I38" t="inlineStr">
-        <is>
-          <t>11:00:00</t>
-        </is>
-      </c>
-      <c r="J38" t="n">
-        <v>19407.89451851702</v>
-      </c>
-      <c r="K38" t="n">
-        <v>0.0601009191845674</v>
-      </c>
-      <c r="L38" t="n">
-        <v>0.05190533929576276</v>
-      </c>
-      <c r="M38" t="inlineStr"/>
-      <c r="N38" t="inlineStr">
-        <is>
-          <t>12:30:00</t>
-        </is>
-      </c>
-      <c r="O38" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="P38" t="inlineStr">
-        <is>
-          <t>15:30:00</t>
-        </is>
-      </c>
-      <c r="Q38" t="n">
-        <v>7110000</v>
-      </c>
-      <c r="R38" t="inlineStr">
-        <is>
-          <t>Consumer Cyclical</t>
-        </is>
-      </c>
-      <c r="S38" t="n">
-        <v>99180000</v>
-      </c>
-      <c r="T38" t="inlineStr">
-        <is>
-          <t>7.11M</t>
-        </is>
-      </c>
-      <c r="U38" t="inlineStr">
-        <is>
-          <t>99.18M</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="1" t="n">
-        <v>29</v>
-      </c>
-      <c r="B39" t="n">
-        <v>0</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>45603</v>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>MTC</t>
-        </is>
-      </c>
-      <c r="E39" t="n">
-        <v>0.4085680272071643</v>
-      </c>
-      <c r="F39" t="n">
-        <v>23.30572258767505</v>
-      </c>
-      <c r="G39" t="n">
-        <v>0.180327868852459</v>
-      </c>
-      <c r="H39" t="n">
-        <v>0.3868</v>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>09:30:00</t>
-        </is>
-      </c>
-      <c r="J39" t="n">
-        <v>2595.389089176887</v>
-      </c>
-      <c r="K39" t="n">
-        <v>0.4494248299278808</v>
-      </c>
-      <c r="L39" t="n">
-        <v>0.3881396258468061</v>
-      </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr">
-        <is>
-          <t>12:30:00</t>
-        </is>
-      </c>
-      <c r="O39" t="inlineStr">
-        <is>
-          <t>10:30:00</t>
-        </is>
-      </c>
-      <c r="P39" t="inlineStr">
-        <is>
-          <t>15:30:00</t>
-        </is>
-      </c>
-      <c r="Q39" t="n">
-        <v>77110000</v>
-      </c>
-      <c r="R39" t="inlineStr">
-        <is>
-          <t>Technology</t>
-        </is>
-      </c>
-      <c r="S39" t="n">
-        <v>198780000</v>
-      </c>
-      <c r="T39" t="inlineStr">
-        <is>
           <t>77.11M</t>
         </is>
       </c>
-      <c r="U39" t="inlineStr">
+      <c r="V36" t="inlineStr">
         <is>
           <t>198.78M</t>
         </is>

</xml_diff>